<commit_message>
feat(export): org documentation, part c2: custom metadata records, opt-in per type
Every sync lists the org's custom metadata types, never their records.
Records are read only for the types an engagement admin turns on in
Privacy & Data (audit-logged), from the next sync; turning a type off
deletes its stored records straight away. New Privacy & Data card (first
10 types, View all to a paged list), GET/PUT /orgs/{id}/custom-metadata,
and two workbook sheets (35 in all). Lumenvale part 11: 4 types, all off by
default. Trust doc updated; no new permission; runbook numbers unchanged.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/samples/lumenvale-org-documentation.xlsx
+++ b/docs/samples/lumenvale-org-documentation.xlsx
@@ -40,6 +40,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Static Resources" sheetId="31" state="visible" r:id="rId31"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Custom Permissions" sheetId="32" state="visible" r:id="rId32"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External Data Sources" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Custom Metadata Types" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Custom Metadata Records" sheetId="35" state="visible" r:id="rId35"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Objects'!$A$1:$L$30</definedName>
@@ -74,6 +76,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="30" hidden="1">'Static Resources'!$A$1:$F$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="31" hidden="1">'Custom Permissions'!$A$1:$F$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="32" hidden="1">'External Data Sources'!$A$1:$F$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="33" hidden="1">'Custom Metadata Types'!$A$1:$C$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="34" hidden="1">'Custom Metadata Records'!$A$1:$F$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -84,7 +88,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -94,6 +98,9 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -121,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -133,6 +140,7 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -498,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -537,7 +545,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 02:52 UTC</t>
+          <t>2026-10-20 02:59 UTC</t>
         </is>
       </c>
     </row>
@@ -561,7 +569,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 02:52 UTC</t>
+          <t>2026-10-20 02:59 UTC</t>
         </is>
       </c>
     </row>
@@ -573,7 +581,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 02:52 UTC</t>
+          <t>2026-10-20 02:59 UTC</t>
         </is>
       </c>
     </row>
@@ -633,7 +641,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 02:52 UTC</t>
+          <t>2026-10-20 02:59 UTC</t>
         </is>
       </c>
     </row>
@@ -652,22 +660,34 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Not included yet</t>
+          <t>Custom metadata</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Custom metadata records, and approval process entry criteria and approvers (they need the Metadata API, which isn't confirmed to work with Newton's permissions).</t>
+          <t>Records are read only for the types an admin turned on for this org (Privacy &amp; Data); the Custom Metadata Types sheet says which.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
+          <t>Not included yet</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Approval process entry criteria and approvers (they need the Metadata API, which isn't confirmed to work with Newton's permissions).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
           <t>Note</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>2 fields aren't visible to the integration user (field-level security), so the describe left them out: their type comes from FieldDefinition; encryption, formula text and picklist values aren't known for them.</t>
         </is>
@@ -61460,6 +61480,173 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:F3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Records</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Discount_Threshold__mdt</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Discount Threshold</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Not read: an admin can turn this type on in Privacy &amp; Data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Feature_Switch__mdt</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Feature Switch</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Not read: an admin can turn this type on in Privacy &amp; Data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Integration_Endpoint__mdt</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Integration Endpoint</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Not read: an admin can turn this type on in Privacy &amp; Data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Region_Mapping__mdt</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Region Mapping</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Not read: an admin can turn this type on in Privacy &amp; Data.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C5"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Namespace</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>No custom metadata records: no type is turned on, or none was read yet.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(export): change history sheet; Change-Risk Radar on demo orgs (item 14)
The Org documentation workbook gains a Change History sheet: every Setup
Audit Trail event Change-Risk Radar has pulled, each once across pulls, with
blast radius and tier, and an About line on range, retention and what the
trail doesn't hold. Change-Risk Radar now runs on demo orgs from the
fixture's audit trail; Lumenvale part 13 adds 60 synthetic changes with
planted risks. Runbook numbers unchanged.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/samples/lumenvale-org-documentation.xlsx
+++ b/docs/samples/lumenvale-org-documentation.xlsx
@@ -43,6 +43,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Custom Metadata Types" sheetId="34" state="visible" r:id="rId34"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Custom Metadata Records" sheetId="35" state="visible" r:id="rId35"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cleanup Candidates" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change History" sheetId="37" state="visible" r:id="rId37"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Objects'!$A$1:$L$30</definedName>
@@ -80,6 +81,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="33" hidden="1">'Custom Metadata Types'!$A$1:$C$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="34" hidden="1">'Custom Metadata Records'!$A$1:$F$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="35" hidden="1">'Cleanup Candidates'!$A$1:$I$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="36" hidden="1">'Change History'!$A$1:$H$61</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -130,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -143,6 +145,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -508,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -547,7 +550,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 03:36 UTC</t>
+          <t>2026-10-20 03:43 UTC</t>
         </is>
       </c>
     </row>
@@ -571,7 +574,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 03:36 UTC</t>
+          <t>2026-10-20 03:43 UTC</t>
         </is>
       </c>
     </row>
@@ -583,7 +586,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 03:36 UTC</t>
+          <t>2026-10-20 03:43 UTC</t>
         </is>
       </c>
     </row>
@@ -643,7 +646,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20 03:36 UTC</t>
+          <t>2026-10-20 03:43 UTC</t>
         </is>
       </c>
     </row>
@@ -692,6 +695,18 @@
       <c r="B15" s="2" t="inlineStr">
         <is>
           <t>2 fields aren't visible to the integration user (field-level security), so the describe left them out: their type comes from FieldDefinition; encryption, formula text and picklist values aren't known for them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>Change history</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>60 Setup Audit Trail events from 2026-09-20 to 2026-10-20, from 1 Change-Risk Radar pull. Salesforce keeps the audit trail for at least 180 days; Newton keeps what it pulled, under its retention settings, so older pulls extend it. The trail doesn't record a field's old and new values.</t>
         </is>
       </c>
     </row>
@@ -64894,6 +64909,2237 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:I79"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H61"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>When (UTC)</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Changed by</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>On behalf of</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Blast radius</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-10-20 00:02</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Manage Users</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>changedUserEmail</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Changed email for user Priya Raman</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Idris Castellan</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-19 23:15</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Manage Permission Sets</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>PermSetAssign</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Permission set Quote Manager: assigned to user Tobias Lindqvist</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Callum Yarrow</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-18 03:53</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Package Manager</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>uninstalledPackage</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Uninstalled package Legacy Survey Tool, permanently deleted its data</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Odette Fennimore</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-17 17:56</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Company Information</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>changedOrgTimeZone</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Changed default time zone</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Nikhil Pemberton</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-16 23:27</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Custom Metadata</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>changedCustomMetadataRecord</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Changed Discount Threshold record Strategic</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Odette Fennimore</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-16 17:13</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Field-Level Security</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>changedFieldSecurity</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Changed field-level security for Compensation Salary Band</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Nikhil Pemberton</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" s="8" t="n">
+        <v>75</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-10-16 13:52</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Custom Metadata</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>changedCustomMetadataRecord</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Changed Discount Threshold record Strategic</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Odette Fennimore</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-10-15 15:52</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Manage Users</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>changedUserEmail</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Changed email for user Elin Sorensen</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Odette Fennimore</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-10-14 19:50</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Flows</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>activatedinteractiondefversion</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Activated flow version Case Triage, version 4</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Ayla Zielinski</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10-13 19:43</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Manage Profiles</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>profileFlsChanged</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Changed profile Sales Rep: field-level security for Account Tax ID</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Callum Yarrow</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-10-13 14:27</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Manage Users</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>deactivateduser</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Deactivated user Tobias Lindqvist</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Odette Fennimore</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-10-12 18:38</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Custom Objects</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>changedCFLength</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Changed field length for Invoice PO Number from 20 to 30</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Marlow Sallow</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-10-12 17:21</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Flows</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>activatedinteractiondefversion</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Activated flow version Case Triage, version 4</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Callum Yarrow</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-10-11 19:02</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Custom Objects</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>changedCFLength</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Changed field length for Invoice PO Number from 20 to 30</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Odette Fennimore</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-10-10 22:03</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Flows</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>deactivatedinteractiondefversion</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Deactivated flow version Legacy Fax Sync, version 3</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Ayla Zielinski</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10-10 21:12</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Customize Accounts</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>changedPicklistValue</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Changed Account Industry picklist value Biotech to Life Sciences</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Nikhil Pemberton</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-07 22:18</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Custom Metadata</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>changedCustomMetadataRecord</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Changed Discount Threshold record Strategic</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Callum Yarrow</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-07 19:44</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Manage Permission Sets</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>PermSetUnassign</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Permission set Lead Conversion: unassigned from user Priya Raman</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Callum Yarrow</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-07 14:48</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Validation Rules</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>newValidationRule</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Created validation rule Old_Score_Range on Account</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Idris Castellan</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-10-07 14:45</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Manage Users</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>createduser</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Created new user Noor Whitlock</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Marlow Sallow</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-06 21:00</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Customize Opportunities</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>createdCFRecordTypeLayout</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Changed page layout assignment for Opportunity Renewal</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Callum Yarrow</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-06 19:51</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Customize Opportunities</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>createdCFRecordTypeLayout</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Changed page layout assignment for Opportunity Renewal</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Odette Fennimore</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-06 15:38</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Manage Users</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>changedUserEmail</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Changed email for user Noor Whitlock</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Idris Castellan</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-10-05 23:14</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Manage Users</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>resetPassword</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Reset password for Priya Raman</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Idris Castellan</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-10-05 18:12</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Flows</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>activatedinteractiondefversion</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Activated flow version Case Triage, version 4</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Nikhil Pemberton</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-10-04 23:53</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Custom Objects</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>changedCFLength</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Changed field length for Invoice PO Number from 20 to 30</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Nikhil Pemberton</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-10-04 21:11</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Manage Permission Sets</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>PermSetAssign</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Permission set Discount Approvals: assigned to user Jun Jovanovic</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Freya Marchetti</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-10-04 21:07</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Manage Permission Sets</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>PermSetAssign</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Permission set Discount Approvals: assigned to user Noor Whitlock</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Freya Marchetti</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-10-04 21:03</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Manage Permission Sets</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>PermSetAssign</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Permission set Discount Approvals: assigned to user Elin Sorensen</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Freya Marchetti</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-10-04 20:59</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Manage Permission Sets</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>PermSetAssign</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Permission set Discount Approvals: assigned to user Mateo Varga</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Freya Marchetti</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-10-04 20:55</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Manage Permission Sets</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>PermSetAssign</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Permission set Discount Approvals: assigned to user Priya Raman</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Freya Marchetti</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-10-04 20:51</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Manage Permission Sets</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>PermSetAssign</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Permission set Discount Approvals: assigned to user Tobias Lindqvist</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Freya Marchetti</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-10-04 20:51</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Custom Objects</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>changedCFLength</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Changed field length for Invoice PO Number from 20 to 30</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Nikhil Pemberton</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-10-04 20:47</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Manage Permission Sets</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>PermSetAssign</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Permission set Discount Approvals: assigned to user Jun Jovanovic</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Freya Marchetti</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-10-04 20:43</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Manage Permission Sets</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>PermSetAssign</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Permission set Discount Approvals: assigned to user Noor Whitlock</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Freya Marchetti</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-10-03 00:25</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Manage Permission Sets</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>PermSetAssign</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Permission set Quote Manager: assigned to user Noor Whitlock</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Idris Castellan</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-10-01 21:40</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Apex Class</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>changedApexClass</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Changed Class code: InvoiceService</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Ayla Zielinski</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-09-30 15:58</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Sharing Defaults</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>changedSharingDefault</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Changed Opportunity organization-wide default from Private to Public Read Only</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Viktor Hawthorne</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>ayla.zielinski@lumenvale.example.com</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="n">
+        <v>75</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-09-29 22:13</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Custom Metadata</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>changedCustomMetadataRecord</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Changed Discount Threshold record Strategic</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Marlow Sallow</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-09-29 17:06</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Customize Opportunities</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>createdCFRecordTypeLayout</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Changed page layout assignment for Opportunity Renewal</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Nikhil Pemberton</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-09-29 14:50</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Apex Class</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>changedApexClass</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Changed Class code: InvoiceService</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Callum Yarrow</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-09-28 17:00</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Customize Opportunities</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>createdCFRecordTypeLayout</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Changed page layout assignment for Opportunity Renewal</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Odette Fennimore</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-09-28 15:20</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Apex Class</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>changedApexClass</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Changed Class code: InvoiceService</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Callum Yarrow</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-09-27 18:19</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Customize Opportunities</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>createdCFRecordTypeLayout</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Changed page layout assignment for Opportunity Renewal</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Viktor Hawthorne</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-09-26 18:45</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Custom Objects</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>changedCFLength</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Changed field length for Invoice PO Number from 20 to 30</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Idris Castellan</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-09-26 18:01</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Email Administration</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>changedEmailDeliverability</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Changed email deliverability to All email</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Ayla Zielinski</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-09-25 18:48</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Manage Permission Sets</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>PermSetAssign</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Permission set Quote Manager: assigned to user Jun Jovanovic</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Ayla Zielinski</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-09-25 14:59</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Manage Users</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>createduser</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Created new user Tobias Lindqvist</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Callum Yarrow</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-09-24 21:28</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Custom Objects</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>changedCFLength</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Changed field length for Invoice PO Number from 20 to 30</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Viktor Hawthorne</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-09-24 18:15</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Manage Permission Sets</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>PermSetAssign</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Permission set Quote Manager: assigned to user Noor Whitlock</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Ayla Zielinski</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-09-24 18:06</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Custom Metadata</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>changedCustomMetadataRecord</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Changed Discount Threshold record Strategic</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Idris Castellan</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-09-24 14:59</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Email Administration</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>changedEmailDeliverability</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Changed email deliverability to All email</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Callum Yarrow</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-09-24 05:23</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Connected Apps</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>insertedConnectedApplication</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Installed connected app DataBridge Sync (package install)</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Marlow Sallow</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" s="8" t="n">
+        <v>95</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-09-23 15:00</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Manage Permission Sets</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>PermSetAssign</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Permission set Quote Manager: assigned to user Noor Whitlock</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Ayla Zielinski</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-09-23 14:59</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Customize Opportunities</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>createdCFRecordTypeLayout</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Changed page layout assignment for Opportunity Renewal</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Nikhil Pemberton</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-09-23 00:35</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Manage Permission Sets</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>PermSetUnassign</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Permission set Lead Conversion: unassigned from user Mateo Varga</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Viktor Hawthorne</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" s="8" t="n">
+        <v>65</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-09-22 18:46</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Flows</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>activatedinteractiondefversion</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Activated flow version Case Triage, version 4</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Ayla Zielinski</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" s="8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-09-22 15:30</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Company Information</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>changedOrgTimeZone</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Changed default time zone</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Freya Marchetti</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" s="8" t="n">
+        <v>40</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-09-21 22:52</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Manage Users</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>changedUserEmail</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Changed email for user Priya Raman</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Freya Marchetti</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-09-20 22:45</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Manage Users</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>createduser</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Created new user Priya Raman</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Nikhil Pemberton</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>